<commit_message>
Daily EOD data and reports for 2026-09-07
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260907.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260907.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.9</v>
+        <v>1.91</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-0.52%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>291043.9</v>
+        <v>292575.71</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-1531.81</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.445</v>
+        <v>2.44</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.035</v>
+        <v>-0.04</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-1.41%</t>
+          <t>-1.61%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>171150</v>
+        <v>170800</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-2450</v>
+        <v>-2800</v>
       </c>
     </row>
     <row r="6">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>63.16</v>
+        <v>62.93</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.91</v>
+        <v>0.68</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.46%</t>
+          <t>1.09%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>505280</v>
+        <v>503440</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>7280</v>
+        <v>5440</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>161.02</v>
+        <v>161.54</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.6</v>
+        <v>1.12</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.37%</t>
+          <t>0.70%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.98</v>
+        <v>0.975</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0</v>
+        <v>-0.005</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-0.51%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>9800</v>
+        <v>9750</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0</v>
+        <v>-50</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>173.41</v>
+        <v>173.18</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-1.09</v>
+        <v>-1.32</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.62%</t>
+          <t>-0.76%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>693640</v>
+        <v>692720</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-4360</v>
+        <v>-5280</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.27</v>
+        <v>0.275</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.89%</t>
+          <t>3.77%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>5400</v>
+        <v>5500</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>34.915</v>
+        <v>35.02</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.045</v>
+        <v>0.06</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.13%</t>
+          <t>0.17%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.205</v>
+        <v>32.33</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.375</v>
+        <v>0.5</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.18%</t>
+          <t>1.57%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>41480.04</v>
+        <v>41641.04</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>483</v>
+        <v>644</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1719672.77</v>
+        <v>1718305.58</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-1872.81</v>
+        <v>-3240</v>
       </c>
     </row>
   </sheetData>

</xml_diff>